<commit_message>
Update CdaToBooleanConceptMap for boolean mapping 468607a5df5dfd691474d575c4e8c19696d445a9
</commit_message>
<xml_diff>
--- a/fsh/ig/CdaToBooleanConceptMap.xlsx
+++ b/fsh/ig/CdaToBooleanConceptMap.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-13T09:40:13+00:00</t>
+    <t>2026-04-13T09:48:02+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -120,7 +120,7 @@
     <t>equivalent</t>
   </si>
   <si>
-    <t>boolean.value</t>
+    <t>boolean</t>
   </si>
 </sst>
 </file>

</xml_diff>